<commit_message>
Delete all Grading Score in all page(Delete grade page)
</commit_message>
<xml_diff>
--- a/test-artifacts/Nursing_Manual_Test_success.xlsx
+++ b/test-artifacts/Nursing_Manual_Test_success.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guton\Desktop\NurseProject\Project-Nurse-main\test-artifacts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F7EC4FF-4E13-4D7D-B811-3801C10FAC85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B6A8B7-1869-4A5B-A039-6FB9AF2067D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="วิธีใช้ + วิธีเปิดหน้า" sheetId="1" r:id="rId1"/>
@@ -713,21 +713,22 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -741,7 +742,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="ปกติ" xfId="0" builtinId="0"/>
@@ -1103,67 +1103,67 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="20.399999999999999" x14ac:dyDescent="0.35">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B3" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
+      <c r="B3" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
     </row>
     <row r="5" spans="2:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
     </row>
     <row r="11" spans="2:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
@@ -1276,11 +1276,11 @@
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -1311,13 +1311,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
@@ -1337,13 +1337,13 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
     </row>
     <row r="4" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
@@ -1453,13 +1453,13 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
     </row>
     <row r="12" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
@@ -1572,13 +1572,13 @@
       <c r="E19" s="19"/>
     </row>
     <row r="20" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="15" t="s">
+      <c r="A20" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="B20" s="16"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
     </row>
     <row r="21" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
@@ -1671,13 +1671,13 @@
       <c r="E26" s="2"/>
     </row>
     <row r="27" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="17" t="s">
+      <c r="A27" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="B27" s="16"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
     </row>
     <row r="28" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
@@ -1774,13 +1774,13 @@
       </c>
     </row>
     <row r="34" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="17" t="s">
+      <c r="A34" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="B34" s="16"/>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
+      <c r="B34" s="17"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
     </row>
     <row r="35" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
@@ -1903,13 +1903,13 @@
       <c r="E42" s="2"/>
     </row>
     <row r="43" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="17" t="s">
+      <c r="A43" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="B43" s="16"/>
-      <c r="C43" s="16"/>
-      <c r="D43" s="16"/>
-      <c r="E43" s="16"/>
+      <c r="B43" s="17"/>
+      <c r="C43" s="17"/>
+      <c r="D43" s="17"/>
+      <c r="E43" s="17"/>
     </row>
     <row r="44" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
@@ -1996,13 +1996,13 @@
       <c r="E49" s="19"/>
     </row>
     <row r="50" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="17" t="s">
+      <c r="A50" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="B50" s="16"/>
-      <c r="C50" s="16"/>
-      <c r="D50" s="16"/>
-      <c r="E50" s="16"/>
+      <c r="B50" s="17"/>
+      <c r="C50" s="17"/>
+      <c r="D50" s="17"/>
+      <c r="E50" s="17"/>
     </row>
     <row r="51" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
@@ -2119,13 +2119,13 @@
       <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="17" t="s">
+      <c r="A59" s="16" t="s">
         <v>133</v>
       </c>
-      <c r="B59" s="16"/>
-      <c r="C59" s="16"/>
-      <c r="D59" s="16"/>
-      <c r="E59" s="16"/>
+      <c r="B59" s="17"/>
+      <c r="C59" s="17"/>
+      <c r="D59" s="17"/>
+      <c r="E59" s="17"/>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="5">
@@ -2185,7 +2185,7 @@
       <c r="D63" s="5">
         <v>1</v>
       </c>
-      <c r="E63" s="25" t="s">
+      <c r="E63" s="13" t="s">
         <v>161</v>
       </c>
     </row>
@@ -2212,13 +2212,13 @@
       <c r="E65" s="19"/>
     </row>
     <row r="66" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="17" t="s">
+      <c r="A66" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="B66" s="16"/>
-      <c r="C66" s="16"/>
-      <c r="D66" s="16"/>
-      <c r="E66" s="16"/>
+      <c r="B66" s="17"/>
+      <c r="C66" s="17"/>
+      <c r="D66" s="17"/>
+      <c r="E66" s="17"/>
     </row>
     <row r="67" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A67" s="5">

</xml_diff>